<commit_message>
Update SplitMap.xlsx and ThePerfectStrangers.rpp with new configurations and data adjustments
</commit_message>
<xml_diff>
--- a/InputList/FullBand/SplitMap.xlsx
+++ b/InputList/FullBand/SplitMap.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="X:\TechnicalDocumentation\Input List\Full Band\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Dev\TechnicalDocumentation\InputList\FullBand\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53F0A2D8-C930-4E22-A947-26C54A4A4F45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99321CB4-E9B0-4EF7-8A2E-C899BD056921}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{976BA9A3-41FE-45E5-BC0B-B40312D9AF21}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" activeTab="1" xr2:uid="{976BA9A3-41FE-45E5-BC0B-B40312D9AF21}"/>
   </bookViews>
   <sheets>
     <sheet name="Split Map" sheetId="3" r:id="rId1"/>
+    <sheet name="Output Map" sheetId="4" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="45">
   <si>
     <t>Top</t>
   </si>
@@ -140,13 +141,65 @@
   </si>
   <si>
     <t>Vocals 7 DCR</t>
+  </si>
+  <si>
+    <t>Billy IEM
+Left</t>
+  </si>
+  <si>
+    <t>Billy IEM
+Right</t>
+  </si>
+  <si>
+    <t>Jessica IEM
+Left</t>
+  </si>
+  <si>
+    <t>Jessica IEM
+Right</t>
+  </si>
+  <si>
+    <t>Paul IEM
+Left</t>
+  </si>
+  <si>
+    <t>Paul IEM
+Right</t>
+  </si>
+  <si>
+    <t>Kenzi IEM
+Left</t>
+  </si>
+  <si>
+    <t>Kenzi IEM
+Right</t>
+  </si>
+  <si>
+    <t>Mike IEM
+Left</t>
+  </si>
+  <si>
+    <t>Mike IEM
+Right</t>
+  </si>
+  <si>
+    <t>Wedge 1</t>
+  </si>
+  <si>
+    <t>Wedge 2</t>
+  </si>
+  <si>
+    <t>Wedge 3</t>
+  </si>
+  <si>
+    <t>Wedge 4</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -216,8 +269,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="12">
+  <fills count="14">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -281,6 +340,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFF00FF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF8181"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="-0.249977111117893"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -365,7 +436,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -432,6 +503,10 @@
     <xf numFmtId="0" fontId="1" fillId="10" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -441,8 +516,13 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -774,35 +854,35 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{728856F4-176B-4634-AD3E-524669928A0A}">
   <dimension ref="A1:Q11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="17" width="12.7109375" customWidth="1"/>
-    <col min="18" max="22" width="14.5703125" customWidth="1"/>
+    <col min="1" max="17" width="12.7265625" customWidth="1"/>
+    <col min="18" max="22" width="14.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="25" t="s">
+    <row r="1" spans="1:17" ht="45" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="27" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
-      <c r="E1" s="26"/>
-      <c r="F1" s="26"/>
-      <c r="G1" s="26"/>
-      <c r="H1" s="26"/>
-      <c r="J1" s="25" t="s">
+      <c r="B1" s="28"/>
+      <c r="C1" s="28"/>
+      <c r="D1" s="28"/>
+      <c r="E1" s="28"/>
+      <c r="F1" s="28"/>
+      <c r="G1" s="28"/>
+      <c r="H1" s="28"/>
+      <c r="J1" s="27" t="s">
         <v>0</v>
       </c>
-      <c r="K1" s="26"/>
-      <c r="L1" s="26"/>
-      <c r="M1" s="26"/>
-      <c r="N1" s="26"/>
-      <c r="O1" s="26"/>
-      <c r="P1" s="26"/>
-      <c r="Q1" s="26"/>
-    </row>
-    <row r="2" spans="1:17" ht="45" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K1" s="28"/>
+      <c r="L1" s="28"/>
+      <c r="M1" s="28"/>
+      <c r="N1" s="28"/>
+      <c r="O1" s="28"/>
+      <c r="P1" s="28"/>
+      <c r="Q1" s="28"/>
+    </row>
+    <row r="2" spans="1:17" ht="45" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A2" s="17">
         <v>1</v>
       </c>
@@ -852,7 +932,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:17" ht="45" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:17" ht="45" customHeight="1" thickTop="1" x14ac:dyDescent="0.45">
       <c r="A3" s="11" t="s">
         <v>10</v>
       </c>
@@ -896,14 +976,14 @@
       <c r="O3" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="P3" s="28" t="s">
+      <c r="P3" s="25" t="s">
         <v>29</v>
       </c>
-      <c r="Q3" s="28" t="s">
+      <c r="Q3" s="25" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="4" spans="1:17" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:17" ht="45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="8" t="s">
         <v>25</v>
       </c>
@@ -929,29 +1009,29 @@
       <c r="P4" s="8"/>
       <c r="Q4" s="8"/>
     </row>
-    <row r="5" spans="1:17" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="25" t="s">
+    <row r="5" spans="1:17" ht="45" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="27" t="s">
         <v>1</v>
       </c>
-      <c r="B5" s="26"/>
-      <c r="C5" s="26"/>
-      <c r="D5" s="26"/>
-      <c r="E5" s="26"/>
-      <c r="F5" s="26"/>
-      <c r="G5" s="26"/>
-      <c r="H5" s="26"/>
-      <c r="J5" s="25" t="s">
+      <c r="B5" s="28"/>
+      <c r="C5" s="28"/>
+      <c r="D5" s="28"/>
+      <c r="E5" s="28"/>
+      <c r="F5" s="28"/>
+      <c r="G5" s="28"/>
+      <c r="H5" s="28"/>
+      <c r="J5" s="27" t="s">
         <v>1</v>
       </c>
-      <c r="K5" s="26"/>
-      <c r="L5" s="26"/>
-      <c r="M5" s="26"/>
-      <c r="N5" s="26"/>
-      <c r="O5" s="26"/>
-      <c r="P5" s="26"/>
-      <c r="Q5" s="26"/>
-    </row>
-    <row r="6" spans="1:17" ht="45" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K5" s="28"/>
+      <c r="L5" s="28"/>
+      <c r="M5" s="28"/>
+      <c r="N5" s="28"/>
+      <c r="O5" s="28"/>
+      <c r="P5" s="28"/>
+      <c r="Q5" s="28"/>
+    </row>
+    <row r="6" spans="1:17" ht="45" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A6" s="21">
         <v>17</v>
       </c>
@@ -1001,7 +1081,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="7" spans="1:17" ht="45" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:17" ht="45" customHeight="1" thickTop="1" x14ac:dyDescent="0.4">
       <c r="A7" s="15" t="s">
         <v>9</v>
       </c>
@@ -1034,7 +1114,7 @@
       <c r="P7" s="16"/>
       <c r="Q7" s="16"/>
     </row>
-    <row r="8" spans="1:17" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:17" ht="45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="9" t="s">
         <v>23</v>
       </c>
@@ -1043,7 +1123,7 @@
         <v>22</v>
       </c>
       <c r="D8" s="9"/>
-      <c r="E8" s="27"/>
+      <c r="E8" s="24"/>
       <c r="F8" s="9"/>
       <c r="G8" s="9" t="s">
         <v>21</v>
@@ -1059,7 +1139,7 @@
       <c r="P8" s="9"/>
       <c r="Q8" s="9"/>
     </row>
-    <row r="9" spans="1:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:17" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="4"/>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
@@ -1074,20 +1154,20 @@
       <c r="P9" s="4"/>
       <c r="Q9" s="4"/>
     </row>
-    <row r="10" spans="1:17" ht="57.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="24" t="s">
+    <row r="10" spans="1:17" ht="58" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="26" t="s">
         <v>24</v>
       </c>
-      <c r="B10" s="24"/>
-      <c r="C10" s="24"/>
-      <c r="D10" s="24"/>
-      <c r="E10" s="24"/>
-      <c r="F10" s="24"/>
-      <c r="G10" s="24"/>
-      <c r="H10" s="24"/>
+      <c r="B10" s="26"/>
+      <c r="C10" s="26"/>
+      <c r="D10" s="26"/>
+      <c r="E10" s="26"/>
+      <c r="F10" s="26"/>
+      <c r="G10" s="26"/>
+      <c r="H10" s="26"/>
       <c r="I10" s="6"/>
     </row>
-    <row r="11" spans="1:17" ht="57.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:17" ht="58" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="6"/>
       <c r="B11" s="6"/>
       <c r="C11" s="6"/>
@@ -1109,4 +1189,144 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{854B4CCA-F0FE-4BDF-9BD8-0023EDDB6E66}">
+  <dimension ref="A1:Q4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="17" width="12.7265625" customWidth="1"/>
+    <col min="18" max="22" width="14.54296875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:17" ht="45" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="20">
+        <v>1</v>
+      </c>
+      <c r="B1" s="20">
+        <v>2</v>
+      </c>
+      <c r="C1" s="20">
+        <v>3</v>
+      </c>
+      <c r="D1" s="20">
+        <v>4</v>
+      </c>
+      <c r="E1" s="20">
+        <v>5</v>
+      </c>
+      <c r="F1" s="20">
+        <v>6</v>
+      </c>
+      <c r="G1" s="20">
+        <v>7</v>
+      </c>
+      <c r="H1" s="20">
+        <v>8</v>
+      </c>
+      <c r="J1" s="20">
+        <v>9</v>
+      </c>
+      <c r="K1" s="20">
+        <v>10</v>
+      </c>
+      <c r="L1" s="20">
+        <v>11</v>
+      </c>
+      <c r="M1" s="20">
+        <v>12</v>
+      </c>
+      <c r="N1" s="20">
+        <v>13</v>
+      </c>
+      <c r="O1" s="20">
+        <v>14</v>
+      </c>
+      <c r="P1" s="20">
+        <v>15</v>
+      </c>
+      <c r="Q1" s="20">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" ht="45" customHeight="1" thickTop="1" x14ac:dyDescent="0.45">
+      <c r="A2" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="B2" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="C2" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="D2" s="13" t="s">
+        <v>34</v>
+      </c>
+      <c r="E2" s="14" t="s">
+        <v>35</v>
+      </c>
+      <c r="F2" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="G2" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="H2" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="I2" s="2"/>
+      <c r="J2" s="31" t="s">
+        <v>39</v>
+      </c>
+      <c r="K2" s="31" t="s">
+        <v>40</v>
+      </c>
+      <c r="L2" s="29" t="s">
+        <v>41</v>
+      </c>
+      <c r="M2" s="29" t="s">
+        <v>42</v>
+      </c>
+      <c r="N2" s="29" t="s">
+        <v>43</v>
+      </c>
+      <c r="O2" s="29" t="s">
+        <v>44</v>
+      </c>
+      <c r="P2" s="30"/>
+      <c r="Q2" s="30"/>
+    </row>
+    <row r="3" spans="1:17" ht="58" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="26" t="s">
+        <v>24</v>
+      </c>
+      <c r="B3" s="26"/>
+      <c r="C3" s="26"/>
+      <c r="D3" s="26"/>
+      <c r="E3" s="26"/>
+      <c r="F3" s="26"/>
+      <c r="G3" s="26"/>
+      <c r="H3" s="26"/>
+      <c r="I3" s="6"/>
+    </row>
+    <row r="4" spans="1:17" ht="58" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="6"/>
+      <c r="B4" s="6"/>
+      <c r="C4" s="6"/>
+      <c r="D4" s="6"/>
+      <c r="E4" s="6"/>
+      <c r="F4" s="6"/>
+      <c r="G4" s="6"/>
+      <c r="H4" s="6"/>
+      <c r="I4" s="1"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A3:H3"/>
+  </mergeCells>
+  <phoneticPr fontId="9" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="landscape" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>